<commit_message>
bug fixed & add instruction
</commit_message>
<xml_diff>
--- a/src/sm/decodetable.xlsx
+++ b/src/sm/decodetable.xlsx
@@ -24308,7 +24308,7 @@
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t>FN_SLTU</t>
+          <t>FN_SLT</t>
         </is>
       </c>
       <c r="Q163" t="inlineStr">
@@ -24455,7 +24455,7 @@
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t>FN_SLTU</t>
+          <t>FN_SLT</t>
         </is>
       </c>
       <c r="Q164" t="inlineStr">

</xml_diff>